<commit_message>
HPO 2048 points without exclusive rule
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_2048_run1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_2048_run1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="521">
   <si>
     <t>Filename</t>
   </si>
@@ -808,769 +808,775 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0.3832,0.1172,0.0929,0.4937</t>
-  </si>
-  <si>
-    <t>0.0083,0.0124,0.0024,0.9912</t>
-  </si>
-  <si>
-    <t>0.6704,0.0290,0.0125,0.3250</t>
-  </si>
-  <si>
-    <t>0.3399,0.0149,0.0240,0.6990</t>
-  </si>
-  <si>
-    <t>0.9952,0.0030,0.0005,0.0013</t>
-  </si>
-  <si>
-    <t>0.9930,0.0035,0.0008,0.0024</t>
-  </si>
-  <si>
-    <t>0.9921,0.0065,0.0011,0.0012</t>
-  </si>
-  <si>
-    <t>0.9944,0.0036,0.0009,0.0010</t>
-  </si>
-  <si>
-    <t>0.9938,0.0047,0.0005,0.0015</t>
-  </si>
-  <si>
-    <t>0.9914,0.0063,0.0012,0.0017</t>
-  </si>
-  <si>
-    <t>0.9946,0.0054,0.0006,0.0007</t>
-  </si>
-  <si>
-    <t>0.9954,0.0024,0.0005,0.0015</t>
-  </si>
-  <si>
-    <t>0.6013,0.1168,0.2688,0.0139</t>
-  </si>
-  <si>
-    <t>0.2043,0.0171,0.8322,0.0130</t>
-  </si>
-  <si>
-    <t>0.2332,0.2148,0.5696,0.0127</t>
-  </si>
-  <si>
-    <t>0.0519,0.6837,0.5305,0.0239</t>
-  </si>
-  <si>
-    <t>0.4974,0.0654,0.4759,0.0475</t>
-  </si>
-  <si>
-    <t>0.0219,0.9648,0.0288,0.0034</t>
-  </si>
-  <si>
-    <t>0.0357,0.9218,0.1234,0.0031</t>
-  </si>
-  <si>
-    <t>0.1729,0.8263,0.0374,0.0092</t>
-  </si>
-  <si>
-    <t>0.1010,0.9041,0.0249,0.0023</t>
-  </si>
-  <si>
-    <t>0.0075,0.9818,0.0372,0.0014</t>
-  </si>
-  <si>
-    <t>0.4615,0.2395,0.2816,0.1592</t>
-  </si>
-  <si>
-    <t>0.3517,0.0899,0.5041,0.1123</t>
-  </si>
-  <si>
-    <t>0.0451,0.0101,0.9445,0.0092</t>
-  </si>
-  <si>
-    <t>0.0609,0.0918,0.8915,0.0166</t>
-  </si>
-  <si>
-    <t>0.1565,0.0705,0.8217,0.0169</t>
-  </si>
-  <si>
-    <t>0.1042,0.0209,0.8219,0.0695</t>
-  </si>
-  <si>
-    <t>0.0119,0.0124,0.9657,0.0209</t>
-  </si>
-  <si>
-    <t>0.1646,0.7810,0.0906,0.0048</t>
-  </si>
-  <si>
-    <t>0.2178,0.2139,0.5911,0.0091</t>
-  </si>
-  <si>
-    <t>0.0127,0.0348,0.9649,0.0271</t>
-  </si>
-  <si>
-    <t>0.0359,0.8325,0.2624,0.0044</t>
-  </si>
-  <si>
-    <t>0.6301,0.1274,0.2343,0.0176</t>
-  </si>
-  <si>
-    <t>0.4397,0.1733,0.4009,0.0427</t>
-  </si>
-  <si>
-    <t>0.4701,0.2553,0.1737,0.0024</t>
-  </si>
-  <si>
-    <t>0.0398,0.8537,0.4036,0.0036</t>
-  </si>
-  <si>
-    <t>0.0162,0.7988,0.5794,0.0550</t>
-  </si>
-  <si>
-    <t>0.0086,0.0364,0.8547,0.2384</t>
-  </si>
-  <si>
-    <t>0.0170,0.7171,0.8574,0.0254</t>
-  </si>
-  <si>
-    <t>0.0166,0.0246,0.8659,0.2226</t>
-  </si>
-  <si>
-    <t>0.0110,0.6328,0.9139,0.0113</t>
-  </si>
-  <si>
-    <t>0.0086,0.9470,0.2997,0.0074</t>
-  </si>
-  <si>
-    <t>0.0154,0.5127,0.8961,0.0125</t>
-  </si>
-  <si>
-    <t>0.2515,0.1238,0.5189,0.2067</t>
-  </si>
-  <si>
-    <t>0.0054,0.9863,0.0213,0.0033</t>
-  </si>
-  <si>
-    <t>0.0041,0.9800,0.1761,0.0013</t>
-  </si>
-  <si>
-    <t>0.0038,0.9862,0.0734,0.0014</t>
-  </si>
-  <si>
-    <t>0.0037,0.1990,0.9740,0.0118</t>
-  </si>
-  <si>
-    <t>0.0046,0.8225,0.9036,0.0054</t>
-  </si>
-  <si>
-    <t>0.0437,0.0327,0.9376,0.0143</t>
-  </si>
-  <si>
-    <t>0.0951,0.0267,0.9142,0.0051</t>
-  </si>
-  <si>
-    <t>0.0248,0.0914,0.9189,0.0367</t>
-  </si>
-  <si>
-    <t>0.0327,0.3785,0.8307,0.0095</t>
-  </si>
-  <si>
-    <t>0.9864,0.0100,0.0023,0.0022</t>
-  </si>
-  <si>
-    <t>0.9787,0.0106,0.0061,0.0036</t>
-  </si>
-  <si>
-    <t>0.9708,0.0240,0.0065,0.0026</t>
-  </si>
-  <si>
-    <t>0.1667,0.0677,0.7769,0.0521</t>
-  </si>
-  <si>
-    <t>0.9881,0.0095,0.0020,0.0016</t>
-  </si>
-  <si>
-    <t>0.9934,0.0049,0.0009,0.0014</t>
-  </si>
-  <si>
-    <t>0.9894,0.0075,0.0014,0.0022</t>
-  </si>
-  <si>
-    <t>0.0022,0.9824,0.2337,0.0128</t>
-  </si>
-  <si>
-    <t>0.0032,0.6723,0.9557,0.0055</t>
-  </si>
-  <si>
-    <t>0.0075,0.2677,0.9426,0.0153</t>
-  </si>
-  <si>
-    <t>0.0035,0.9591,0.6263,0.0076</t>
-  </si>
-  <si>
-    <t>0.0102,0.1784,0.9549,0.0211</t>
-  </si>
-  <si>
-    <t>0.0183,0.9303,0.1434,0.0039</t>
-  </si>
-  <si>
-    <t>0.0097,0.9868,0.0080,0.0007</t>
-  </si>
-  <si>
-    <t>0.7035,0.0379,0.3280,0.0054</t>
-  </si>
-  <si>
-    <t>0.2831,0.2707,0.4920,0.0163</t>
-  </si>
-  <si>
-    <t>0.0135,0.1462,0.9535,0.0042</t>
-  </si>
-  <si>
-    <t>0.0051,0.9522,0.5358,0.0115</t>
-  </si>
-  <si>
-    <t>0.0138,0.7530,0.8062,0.0143</t>
-  </si>
-  <si>
-    <t>0.0060,0.9633,0.3254,0.0058</t>
-  </si>
-  <si>
-    <t>0.0009,0.9873,0.2949,0.0048</t>
-  </si>
-  <si>
-    <t>0.0818,0.0157,0.0249,0.9271</t>
-  </si>
-  <si>
-    <t>0.0038,0.0088,0.0022,0.9948</t>
-  </si>
-  <si>
-    <t>0.0051,0.0071,0.0019,0.9948</t>
-  </si>
-  <si>
-    <t>0.0048,0.0054,0.0013,0.9957</t>
-  </si>
-  <si>
-    <t>0.0114,0.0100,0.0091,0.9850</t>
-  </si>
-  <si>
-    <t>0.0073,0.0116,0.0088,0.9875</t>
-  </si>
-  <si>
-    <t>0.0027,0.9281,0.8250,0.0036</t>
-  </si>
-  <si>
-    <t>0.0014,0.7362,0.9768,0.0010</t>
-  </si>
-  <si>
-    <t>0.0095,0.8587,0.7932,0.0101</t>
-  </si>
-  <si>
-    <t>0.0065,0.7082,0.9219,0.0066</t>
-  </si>
-  <si>
-    <t>0.0041,0.9468,0.6323,0.0037</t>
-  </si>
-  <si>
-    <t>0.0028,0.9172,0.8437,0.0041</t>
-  </si>
-  <si>
-    <t>0.9929,0.0052,0.0010,0.0014</t>
-  </si>
-  <si>
-    <t>0.9917,0.0071,0.0011,0.0012</t>
-  </si>
-  <si>
-    <t>0.9937,0.0058,0.0010,0.0007</t>
-  </si>
-  <si>
-    <t>0.9906,0.0073,0.0016,0.0015</t>
-  </si>
-  <si>
-    <t>0.9916,0.0068,0.0015,0.0010</t>
-  </si>
-  <si>
-    <t>0.9892,0.0094,0.0019,0.0016</t>
-  </si>
-  <si>
-    <t>0.9893,0.0091,0.0017,0.0014</t>
-  </si>
-  <si>
-    <t>0.9921,0.0069,0.0010,0.0013</t>
-  </si>
-  <si>
-    <t>0.9940,0.0032,0.0007,0.0017</t>
-  </si>
-  <si>
-    <t>0.9924,0.0049,0.0009,0.0020</t>
-  </si>
-  <si>
-    <t>0.9918,0.0037,0.0009,0.0028</t>
-  </si>
-  <si>
-    <t>0.9935,0.0013,0.0003,0.0039</t>
-  </si>
-  <si>
-    <t>0.9937,0.0048,0.0007,0.0012</t>
-  </si>
-  <si>
-    <t>0.9867,0.0098,0.0025,0.0020</t>
-  </si>
-  <si>
-    <t>0.9930,0.0042,0.0009,0.0021</t>
-  </si>
-  <si>
-    <t>0.9912,0.0047,0.0016,0.0020</t>
-  </si>
-  <si>
-    <t>0.0045,0.0141,0.9881,0.0097</t>
-  </si>
-  <si>
-    <t>0.0124,0.0309,0.9679,0.0180</t>
-  </si>
-  <si>
-    <t>0.5849,0.0950,0.3568,0.0941</t>
-  </si>
-  <si>
-    <t>0.0604,0.0302,0.8887,0.0391</t>
-  </si>
-  <si>
-    <t>0.0563,0.9305,0.0279,0.0083</t>
-  </si>
-  <si>
-    <t>0.0457,0.9394,0.0310,0.0044</t>
-  </si>
-  <si>
-    <t>0.5973,0.4671,0.0256,0.0035</t>
-  </si>
-  <si>
-    <t>0.4677,0.4982,0.0455,0.0025</t>
-  </si>
-  <si>
-    <t>0.0745,0.8810,0.0788,0.0066</t>
-  </si>
-  <si>
-    <t>0.0173,0.9693,0.0362,0.0025</t>
-  </si>
-  <si>
-    <t>0.5510,0.3762,0.0709,0.0050</t>
-  </si>
-  <si>
-    <t>0.4987,0.2456,0.2278,0.0196</t>
-  </si>
-  <si>
-    <t>0.1181,0.0425,0.8681,0.0123</t>
-  </si>
-  <si>
-    <t>0.1784,0.7387,0.0940,0.1379</t>
-  </si>
-  <si>
-    <t>0.5762,0.0894,0.3216,0.0122</t>
-  </si>
-  <si>
-    <t>0.3415,0.4631,0.2906,0.0902</t>
-  </si>
-  <si>
-    <t>0.0036,0.9862,0.0828,0.0009</t>
-  </si>
-  <si>
-    <t>0.0041,0.9870,0.0618,0.0015</t>
-  </si>
-  <si>
-    <t>0.0132,0.9754,0.0149,0.0170</t>
-  </si>
-  <si>
-    <t>0.0008,0.9892,0.3341,0.0005</t>
-  </si>
-  <si>
-    <t>0.0254,0.9163,0.2488,0.0012</t>
-  </si>
-  <si>
-    <t>0.8459,0.1038,0.0489,0.0026</t>
-  </si>
-  <si>
-    <t>0.7601,0.1746,0.0507,0.0020</t>
-  </si>
-  <si>
-    <t>0.9761,0.0169,0.0046,0.0047</t>
-  </si>
-  <si>
-    <t>0.9845,0.0128,0.0028,0.0028</t>
-  </si>
-  <si>
-    <t>0.9848,0.0106,0.0020,0.0032</t>
-  </si>
-  <si>
-    <t>0.9858,0.0047,0.0026,0.0042</t>
-  </si>
-  <si>
-    <t>0.9945,0.0038,0.0006,0.0013</t>
-  </si>
-  <si>
-    <t>0.9481,0.0592,0.0085,0.0031</t>
-  </si>
-  <si>
-    <t>0.9804,0.0108,0.0044,0.0049</t>
-  </si>
-  <si>
-    <t>0.9835,0.0053,0.0021,0.0070</t>
-  </si>
-  <si>
-    <t>0.0052,0.7883,0.9048,0.0074</t>
-  </si>
-  <si>
-    <t>0.0096,0.8379,0.7407,0.0081</t>
-  </si>
-  <si>
-    <t>0.0092,0.6628,0.8919,0.0071</t>
-  </si>
-  <si>
-    <t>0.0116,0.4741,0.9371,0.0105</t>
-  </si>
-  <si>
-    <t>0.6644,0.1809,0.1500,0.0254</t>
-  </si>
-  <si>
-    <t>0.4176,0.4543,0.0798,0.1155</t>
-  </si>
-  <si>
-    <t>0.3519,0.0058,0.5505,0.0663</t>
-  </si>
-  <si>
-    <t>0.4639,0.4946,0.0955,0.0892</t>
-  </si>
-  <si>
-    <t>0.0491,0.0084,0.0121,0.9652</t>
-  </si>
-  <si>
-    <t>0.0006,0.0033,0.0006,0.9987</t>
-  </si>
-  <si>
-    <t>0.0033,0.0187,0.0049,0.9921</t>
-  </si>
-  <si>
-    <t>0.0374,0.0099,0.0066,0.9742</t>
-  </si>
-  <si>
-    <t>0.0027,0.9330,0.8130,0.0057</t>
-  </si>
-  <si>
-    <t>0.9761,0.0148,0.0084,0.0027</t>
-  </si>
-  <si>
-    <t>0.6271,0.4200,0.0300,0.0148</t>
-  </si>
-  <si>
-    <t>0.9711,0.0171,0.0052,0.0089</t>
-  </si>
-  <si>
-    <t>0.9571,0.0306,0.0137,0.0039</t>
-  </si>
-  <si>
-    <t>0.9756,0.0112,0.0057,0.0065</t>
-  </si>
-  <si>
-    <t>0.7243,0.0226,0.0295,0.2402</t>
-  </si>
-  <si>
-    <t>0.9715,0.0069,0.0025,0.0163</t>
-  </si>
-  <si>
-    <t>0.1357,0.6716,0.2390,0.1673</t>
-  </si>
-  <si>
-    <t>0.5126,0.0035,0.0075,0.5892</t>
-  </si>
-  <si>
-    <t>0.8544,0.0096,0.0086,0.1207</t>
-  </si>
-  <si>
-    <t>0.3020,0.6660,0.0620,0.0108</t>
-  </si>
-  <si>
-    <t>0.7864,0.1455,0.0691,0.0081</t>
-  </si>
-  <si>
-    <t>0.7697,0.1657,0.0618,0.0082</t>
-  </si>
-  <si>
-    <t>0.2315,0.7405,0.0760,0.0384</t>
-  </si>
-  <si>
-    <t>0.5181,0.4374,0.0807,0.0146</t>
-  </si>
-  <si>
-    <t>0.6487,0.1951,0.1244,0.0140</t>
-  </si>
-  <si>
-    <t>0.9906,0.0036,0.0010,0.0037</t>
-  </si>
-  <si>
-    <t>0.9915,0.0055,0.0011,0.0021</t>
-  </si>
-  <si>
-    <t>0.9913,0.0063,0.0015,0.0016</t>
-  </si>
-  <si>
-    <t>0.9917,0.0050,0.0012,0.0017</t>
-  </si>
-  <si>
-    <t>0.9871,0.0097,0.0027,0.0020</t>
-  </si>
-  <si>
-    <t>0.9921,0.0048,0.0010,0.0018</t>
-  </si>
-  <si>
-    <t>0.9905,0.0055,0.0013,0.0030</t>
-  </si>
-  <si>
-    <t>0.9901,0.0053,0.0019,0.0023</t>
-  </si>
-  <si>
-    <t>0.5087,0.3830,0.0802,0.0047</t>
-  </si>
-  <si>
-    <t>0.8533,0.2206,0.0101,0.0042</t>
-  </si>
-  <si>
-    <t>0.6985,0.3266,0.0379,0.0112</t>
-  </si>
-  <si>
-    <t>0.5584,0.1220,0.3438,0.0055</t>
-  </si>
-  <si>
-    <t>0.9764,0.0172,0.0054,0.0024</t>
-  </si>
-  <si>
-    <t>0.9338,0.0574,0.0156,0.0043</t>
-  </si>
-  <si>
-    <t>0.9816,0.0192,0.0023,0.0020</t>
-  </si>
-  <si>
-    <t>0.5721,0.4861,0.0260,0.0046</t>
-  </si>
-  <si>
-    <t>0.0111,0.2413,0.9607,0.0043</t>
-  </si>
-  <si>
-    <t>0.9641,0.0448,0.0052,0.0023</t>
-  </si>
-  <si>
-    <t>0.0025,0.0230,0.9920,0.0039</t>
-  </si>
-  <si>
-    <t>0.0017,0.9030,0.9159,0.0031</t>
-  </si>
-  <si>
-    <t>0.0599,0.0503,0.9291,0.0109</t>
-  </si>
-  <si>
-    <t>0.0046,0.2913,0.9775,0.0035</t>
-  </si>
-  <si>
-    <t>0.0054,0.0617,0.9818,0.0071</t>
-  </si>
-  <si>
-    <t>0.0058,0.0073,0.9836,0.0094</t>
-  </si>
-  <si>
-    <t>0.0064,0.1599,0.9722,0.0057</t>
-  </si>
-  <si>
-    <t>0.2588,0.3775,0.4017,0.0319</t>
-  </si>
-  <si>
-    <t>0.2132,0.1505,0.6917,0.0517</t>
-  </si>
-  <si>
-    <t>0.4107,0.3829,0.2845,0.0822</t>
-  </si>
-  <si>
-    <t>0.1244,0.5442,0.3649,0.0185</t>
-  </si>
-  <si>
-    <t>0.0701,0.4679,0.6436,0.0161</t>
-  </si>
-  <si>
-    <t>0.2366,0.4748,0.2516,0.0317</t>
-  </si>
-  <si>
-    <t>0.4829,0.1167,0.3911,0.0233</t>
-  </si>
-  <si>
-    <t>0.4074,0.1008,0.5434,0.0355</t>
-  </si>
-  <si>
-    <t>0.9027,0.1279,0.0128,0.0044</t>
-  </si>
-  <si>
-    <t>0.9564,0.0551,0.0060,0.0027</t>
-  </si>
-  <si>
-    <t>0.9770,0.0251,0.0034,0.0017</t>
-  </si>
-  <si>
-    <t>0.9861,0.0123,0.0026,0.0018</t>
-  </si>
-  <si>
-    <t>0.9541,0.0563,0.0077,0.0023</t>
-  </si>
-  <si>
-    <t>0.0517,0.8868,0.0806,0.0691</t>
-  </si>
-  <si>
-    <t>0.6956,0.0883,0.2206,0.0388</t>
-  </si>
-  <si>
-    <t>0.2594,0.3412,0.1761,0.4056</t>
-  </si>
-  <si>
-    <t>0.1900,0.0434,0.7256,0.0731</t>
-  </si>
-  <si>
-    <t>0.2459,0.2774,0.3020,0.2679</t>
-  </si>
-  <si>
-    <t>0.0315,0.1001,0.8795,0.0890</t>
-  </si>
-  <si>
-    <t>0.0187,0.2892,0.8412,0.0868</t>
-  </si>
-  <si>
-    <t>0.0118,0.0860,0.9483,0.0392</t>
-  </si>
-  <si>
-    <t>0.0252,0.3732,0.9038,0.0282</t>
-  </si>
-  <si>
-    <t>0.0148,0.4174,0.9148,0.0186</t>
-  </si>
-  <si>
-    <t>0.9920,0.0045,0.0009,0.0024</t>
-  </si>
-  <si>
-    <t>0.9922,0.0054,0.0011,0.0015</t>
-  </si>
-  <si>
-    <t>0.9941,0.0048,0.0007,0.0010</t>
-  </si>
-  <si>
-    <t>0.9893,0.0101,0.0013,0.0012</t>
-  </si>
-  <si>
-    <t>0.9888,0.0094,0.0021,0.0012</t>
-  </si>
-  <si>
-    <t>0.9924,0.0068,0.0011,0.0009</t>
-  </si>
-  <si>
-    <t>0.9844,0.0072,0.0018,0.0053</t>
-  </si>
-  <si>
-    <t>0.9933,0.0048,0.0007,0.0016</t>
-  </si>
-  <si>
-    <t>0.2005,0.0582,0.8254,0.0084</t>
-  </si>
-  <si>
-    <t>0.1948,0.6279,0.2181,0.0090</t>
-  </si>
-  <si>
-    <t>0.7741,0.1848,0.0301,0.0570</t>
-  </si>
-  <si>
-    <t>0.0031,0.0577,0.9875,0.0039</t>
-  </si>
-  <si>
-    <t>0.0011,0.0716,0.9913,0.0045</t>
-  </si>
-  <si>
-    <t>0.0242,0.3808,0.8501,0.0251</t>
-  </si>
-  <si>
-    <t>0.0020,0.0949,0.9907,0.0032</t>
-  </si>
-  <si>
-    <t>0.0399,0.3797,0.7746,0.0087</t>
-  </si>
-  <si>
-    <t>0.0042,0.0712,0.9860,0.0070</t>
-  </si>
-  <si>
-    <t>0.0417,0.2497,0.8609,0.0140</t>
-  </si>
-  <si>
-    <t>0.0124,0.9160,0.3541,0.0149</t>
-  </si>
-  <si>
-    <t>0.1287,0.7519,0.1655,0.1297</t>
-  </si>
-  <si>
-    <t>0.5835,0.0418,0.4554,0.0305</t>
-  </si>
-  <si>
-    <t>0.8102,0.0396,0.1144,0.0594</t>
-  </si>
-  <si>
-    <t>0.9858,0.0133,0.0022,0.0018</t>
-  </si>
-  <si>
-    <t>0.9917,0.0062,0.0011,0.0015</t>
-  </si>
-  <si>
-    <t>0.9933,0.0036,0.0008,0.0020</t>
-  </si>
-  <si>
-    <t>0.9856,0.0106,0.0040,0.0016</t>
-  </si>
-  <si>
-    <t>0.9906,0.0064,0.0013,0.0022</t>
-  </si>
-  <si>
-    <t>0.9918,0.0047,0.0014,0.0018</t>
-  </si>
-  <si>
-    <t>0.9895,0.0104,0.0014,0.0012</t>
-  </si>
-  <si>
-    <t>0.9930,0.0054,0.0009,0.0010</t>
-  </si>
-  <si>
-    <t>0.0644,0.3884,0.7683,0.0260</t>
-  </si>
-  <si>
-    <t>0.0045,0.4685,0.9666,0.0039</t>
-  </si>
-  <si>
-    <t>0.0067,0.6364,0.9177,0.0074</t>
-  </si>
-  <si>
-    <t>0.0362,0.7532,0.5146,0.0418</t>
-  </si>
-  <si>
-    <t>0.0172,0.0157,0.9609,0.0176</t>
-  </si>
-  <si>
-    <t>0.0558,0.0304,0.6675,0.3613</t>
-  </si>
-  <si>
-    <t>0.3174,0.0422,0.6706,0.0480</t>
-  </si>
-  <si>
-    <t>0.0159,0.0609,0.8851,0.1517</t>
-  </si>
-  <si>
-    <t>0.4106,0.0307,0.0128,0.6407</t>
-  </si>
-  <si>
-    <t>0.0322,0.0238,0.0086,0.9741</t>
-  </si>
-  <si>
-    <t>0.0285,0.0135,0.0038,0.9796</t>
-  </si>
-  <si>
-    <t>0.0114,0.0022,0.0009,0.9939</t>
-  </si>
-  <si>
-    <t>0.0059,0.0023,0.0011,0.9957</t>
-  </si>
-  <si>
-    <t>0.2534,0.5284,0.0772,0.3380</t>
+    <t>0,0,0,0</t>
+  </si>
+  <si>
+    <t>1,0,1,0</t>
+  </si>
+  <si>
+    <t>0.6027,0.2598,0.1497,0.0399</t>
+  </si>
+  <si>
+    <t>0.0056,0.0052,0.0020,0.9946</t>
+  </si>
+  <si>
+    <t>0.0470,0.0156,0.0051,0.9665</t>
+  </si>
+  <si>
+    <t>0.0468,0.0111,0.0062,0.9686</t>
+  </si>
+  <si>
+    <t>0.9906,0.0028,0.0006,0.0049</t>
+  </si>
+  <si>
+    <t>0.9903,0.0050,0.0007,0.0037</t>
+  </si>
+  <si>
+    <t>0.9915,0.0067,0.0015,0.0012</t>
+  </si>
+  <si>
+    <t>0.9947,0.0025,0.0005,0.0018</t>
+  </si>
+  <si>
+    <t>0.9918,0.0064,0.0010,0.0015</t>
+  </si>
+  <si>
+    <t>0.9928,0.0049,0.0011,0.0016</t>
+  </si>
+  <si>
+    <t>0.9941,0.0032,0.0007,0.0017</t>
+  </si>
+  <si>
+    <t>0.9940,0.0030,0.0008,0.0018</t>
+  </si>
+  <si>
+    <t>0.2168,0.5432,0.2822,0.0282</t>
+  </si>
+  <si>
+    <t>0.0521,0.0932,0.9047,0.0141</t>
+  </si>
+  <si>
+    <t>0.2941,0.1445,0.5920,0.0110</t>
+  </si>
+  <si>
+    <t>0.0461,0.5054,0.7423,0.0183</t>
+  </si>
+  <si>
+    <t>0.6327,0.1049,0.2656,0.0110</t>
+  </si>
+  <si>
+    <t>0.0135,0.9720,0.0548,0.0010</t>
+  </si>
+  <si>
+    <t>0.0379,0.9431,0.0469,0.0029</t>
+  </si>
+  <si>
+    <t>0.4986,0.5202,0.0449,0.0077</t>
+  </si>
+  <si>
+    <t>0.0882,0.8996,0.0318,0.0045</t>
+  </si>
+  <si>
+    <t>0.0179,0.9726,0.0258,0.0015</t>
+  </si>
+  <si>
+    <t>0.6080,0.0578,0.3937,0.0291</t>
+  </si>
+  <si>
+    <t>0.1975,0.0665,0.7136,0.0763</t>
+  </si>
+  <si>
+    <t>0.0466,0.0220,0.9283,0.0184</t>
+  </si>
+  <si>
+    <t>0.1169,0.2217,0.7054,0.0357</t>
+  </si>
+  <si>
+    <t>0.0762,0.0358,0.9224,0.0055</t>
+  </si>
+  <si>
+    <t>0.3191,0.0383,0.7192,0.0155</t>
+  </si>
+  <si>
+    <t>0.0041,0.0144,0.9846,0.0136</t>
+  </si>
+  <si>
+    <t>0.4211,0.5854,0.0380,0.0046</t>
+  </si>
+  <si>
+    <t>0.3838,0.1177,0.5481,0.0091</t>
+  </si>
+  <si>
+    <t>0.0299,0.0442,0.9440,0.0247</t>
+  </si>
+  <si>
+    <t>0.0428,0.8843,0.1366,0.0069</t>
+  </si>
+  <si>
+    <t>0.5667,0.2267,0.2077,0.0330</t>
+  </si>
+  <si>
+    <t>0.3357,0.1844,0.4868,0.0372</t>
+  </si>
+  <si>
+    <t>0.7511,0.1615,0.0537,0.0018</t>
+  </si>
+  <si>
+    <t>0.0416,0.8517,0.3814,0.0049</t>
+  </si>
+  <si>
+    <t>0.0114,0.9182,0.3336,0.0265</t>
+  </si>
+  <si>
+    <t>0.0094,0.1192,0.9549,0.0334</t>
+  </si>
+  <si>
+    <t>0.0149,0.7678,0.8577,0.0212</t>
+  </si>
+  <si>
+    <t>0.0279,0.0165,0.6861,0.4117</t>
+  </si>
+  <si>
+    <t>0.0118,0.4621,0.9146,0.0060</t>
+  </si>
+  <si>
+    <t>0.0050,0.9174,0.6204,0.0065</t>
+  </si>
+  <si>
+    <t>0.0376,0.2101,0.9043,0.0228</t>
+  </si>
+  <si>
+    <t>0.0984,0.3704,0.0538,0.8197</t>
+  </si>
+  <si>
+    <t>0.0025,0.9929,0.0138,0.0023</t>
+  </si>
+  <si>
+    <t>0.0030,0.9891,0.0643,0.0011</t>
+  </si>
+  <si>
+    <t>0.0035,0.9773,0.2672,0.0022</t>
+  </si>
+  <si>
+    <t>0.0033,0.6616,0.9218,0.0103</t>
+  </si>
+  <si>
+    <t>0.0018,0.8377,0.9494,0.0019</t>
+  </si>
+  <si>
+    <t>0.0250,0.1174,0.9459,0.0119</t>
+  </si>
+  <si>
+    <t>0.0897,0.0273,0.9316,0.0029</t>
+  </si>
+  <si>
+    <t>0.0094,0.0503,0.9747,0.0115</t>
+  </si>
+  <si>
+    <t>0.0221,0.0535,0.9648,0.0061</t>
+  </si>
+  <si>
+    <t>0.9715,0.0364,0.0040,0.0015</t>
+  </si>
+  <si>
+    <t>0.9894,0.0066,0.0025,0.0015</t>
+  </si>
+  <si>
+    <t>0.9841,0.0132,0.0027,0.0024</t>
+  </si>
+  <si>
+    <t>0.2359,0.1466,0.6485,0.0236</t>
+  </si>
+  <si>
+    <t>0.9874,0.0076,0.0030,0.0022</t>
+  </si>
+  <si>
+    <t>0.9899,0.0078,0.0013,0.0020</t>
+  </si>
+  <si>
+    <t>0.9814,0.0199,0.0029,0.0019</t>
+  </si>
+  <si>
+    <t>0.0020,0.9825,0.3211,0.0070</t>
+  </si>
+  <si>
+    <t>0.0021,0.4169,0.9788,0.0038</t>
+  </si>
+  <si>
+    <t>0.0130,0.1824,0.9265,0.0160</t>
+  </si>
+  <si>
+    <t>0.0028,0.9051,0.8912,0.0038</t>
+  </si>
+  <si>
+    <t>0.0020,0.0446,0.9887,0.0083</t>
+  </si>
+  <si>
+    <t>0.0217,0.9398,0.1006,0.0049</t>
+  </si>
+  <si>
+    <t>0.0183,0.9821,0.0050,0.0007</t>
+  </si>
+  <si>
+    <t>0.5902,0.0265,0.5380,0.0097</t>
+  </si>
+  <si>
+    <t>0.6851,0.1175,0.2227,0.0211</t>
+  </si>
+  <si>
+    <t>0.0127,0.4088,0.8968,0.0039</t>
+  </si>
+  <si>
+    <t>0.0028,0.9474,0.7175,0.0047</t>
+  </si>
+  <si>
+    <t>0.0039,0.9255,0.7670,0.0055</t>
+  </si>
+  <si>
+    <t>0.0035,0.9841,0.1829,0.0036</t>
+  </si>
+  <si>
+    <t>0.0012,0.9846,0.3950,0.0030</t>
+  </si>
+  <si>
+    <t>0.0096,0.0076,0.0047,0.9905</t>
+  </si>
+  <si>
+    <t>0.0040,0.0085,0.0013,0.9955</t>
+  </si>
+  <si>
+    <t>0.0014,0.0030,0.0012,0.9977</t>
+  </si>
+  <si>
+    <t>0.0152,0.0120,0.0091,0.9838</t>
+  </si>
+  <si>
+    <t>0.0057,0.0063,0.0016,0.9946</t>
+  </si>
+  <si>
+    <t>0.0072,0.0146,0.0021,0.9920</t>
+  </si>
+  <si>
+    <t>0.0026,0.9766,0.4236,0.0063</t>
+  </si>
+  <si>
+    <t>0.0033,0.6356,0.9698,0.0024</t>
+  </si>
+  <si>
+    <t>0.0162,0.6254,0.8239,0.0124</t>
+  </si>
+  <si>
+    <t>0.0048,0.8908,0.7774,0.0168</t>
+  </si>
+  <si>
+    <t>0.0028,0.9554,0.5827,0.0029</t>
+  </si>
+  <si>
+    <t>0.0036,0.9707,0.4288,0.0071</t>
+  </si>
+  <si>
+    <t>0.9955,0.0045,0.0005,0.0005</t>
+  </si>
+  <si>
+    <t>0.9911,0.0070,0.0014,0.0013</t>
+  </si>
+  <si>
+    <t>0.9850,0.0135,0.0027,0.0020</t>
+  </si>
+  <si>
+    <t>0.9883,0.0070,0.0015,0.0039</t>
+  </si>
+  <si>
+    <t>0.9902,0.0091,0.0015,0.0012</t>
+  </si>
+  <si>
+    <t>0.9944,0.0042,0.0005,0.0012</t>
+  </si>
+  <si>
+    <t>0.9904,0.0097,0.0015,0.0010</t>
+  </si>
+  <si>
+    <t>0.9922,0.0055,0.0010,0.0018</t>
+  </si>
+  <si>
+    <t>0.9928,0.0036,0.0006,0.0028</t>
+  </si>
+  <si>
+    <t>0.9940,0.0048,0.0007,0.0010</t>
+  </si>
+  <si>
+    <t>0.9948,0.0027,0.0006,0.0016</t>
+  </si>
+  <si>
+    <t>0.9952,0.0030,0.0006,0.0011</t>
+  </si>
+  <si>
+    <t>0.9931,0.0046,0.0010,0.0016</t>
+  </si>
+  <si>
+    <t>0.9926,0.0056,0.0008,0.0014</t>
+  </si>
+  <si>
+    <t>0.9927,0.0058,0.0008,0.0017</t>
+  </si>
+  <si>
+    <t>0.9910,0.0055,0.0012,0.0021</t>
+  </si>
+  <si>
+    <t>0.0040,0.0165,0.9866,0.0115</t>
+  </si>
+  <si>
+    <t>0.0533,0.0726,0.9145,0.0111</t>
+  </si>
+  <si>
+    <t>0.3756,0.0418,0.4331,0.1826</t>
+  </si>
+  <si>
+    <t>0.1106,0.0375,0.8847,0.0099</t>
+  </si>
+  <si>
+    <t>0.0559,0.9246,0.0445,0.0063</t>
+  </si>
+  <si>
+    <t>0.0426,0.9427,0.0331,0.0027</t>
+  </si>
+  <si>
+    <t>0.3691,0.6993,0.0213,0.0031</t>
+  </si>
+  <si>
+    <t>0.2967,0.6813,0.0476,0.0029</t>
+  </si>
+  <si>
+    <t>0.0237,0.9551,0.0625,0.0035</t>
+  </si>
+  <si>
+    <t>0.0157,0.9718,0.0278,0.0027</t>
+  </si>
+  <si>
+    <t>0.3720,0.6869,0.0266,0.0080</t>
+  </si>
+  <si>
+    <t>0.3889,0.4009,0.1859,0.0168</t>
+  </si>
+  <si>
+    <t>0.1794,0.0188,0.8532,0.0094</t>
+  </si>
+  <si>
+    <t>0.2203,0.6861,0.1329,0.1038</t>
+  </si>
+  <si>
+    <t>0.3447,0.2649,0.3957,0.0284</t>
+  </si>
+  <si>
+    <t>0.2847,0.4810,0.0719,0.3589</t>
+  </si>
+  <si>
+    <t>0.0067,0.9819,0.0576,0.0015</t>
+  </si>
+  <si>
+    <t>0.0056,0.9837,0.0708,0.0019</t>
+  </si>
+  <si>
+    <t>0.0120,0.9721,0.0241,0.0204</t>
+  </si>
+  <si>
+    <t>0.0019,0.9937,0.0443,0.0007</t>
+  </si>
+  <si>
+    <t>0.0165,0.9362,0.2889,0.0012</t>
+  </si>
+  <si>
+    <t>0.6906,0.2197,0.0639,0.0027</t>
+  </si>
+  <si>
+    <t>0.6600,0.2752,0.0641,0.0027</t>
+  </si>
+  <si>
+    <t>0.9776,0.0171,0.0039,0.0032</t>
+  </si>
+  <si>
+    <t>0.9933,0.0036,0.0008,0.0016</t>
+  </si>
+  <si>
+    <t>0.9835,0.0059,0.0020,0.0068</t>
+  </si>
+  <si>
+    <t>0.9840,0.0070,0.0022,0.0050</t>
+  </si>
+  <si>
+    <t>0.9940,0.0049,0.0006,0.0011</t>
+  </si>
+  <si>
+    <t>0.9734,0.0310,0.0041,0.0021</t>
+  </si>
+  <si>
+    <t>0.9838,0.0091,0.0031,0.0039</t>
+  </si>
+  <si>
+    <t>0.9827,0.0077,0.0042,0.0036</t>
+  </si>
+  <si>
+    <t>0.0068,0.8440,0.8328,0.0080</t>
+  </si>
+  <si>
+    <t>0.0109,0.6330,0.8803,0.0065</t>
+  </si>
+  <si>
+    <t>0.0040,0.4131,0.9774,0.0015</t>
+  </si>
+  <si>
+    <t>0.0148,0.3716,0.9330,0.0146</t>
+  </si>
+  <si>
+    <t>0.6950,0.1775,0.1257,0.0453</t>
+  </si>
+  <si>
+    <t>0.7217,0.1381,0.1235,0.0193</t>
+  </si>
+  <si>
+    <t>0.3534,0.0107,0.7530,0.0108</t>
+  </si>
+  <si>
+    <t>0.2941,0.6639,0.0507,0.0925</t>
+  </si>
+  <si>
+    <t>0.0537,0.0116,0.0113,0.9625</t>
+  </si>
+  <si>
+    <t>0.0004,0.0019,0.0009,0.9988</t>
+  </si>
+  <si>
+    <t>0.0103,0.0138,0.0120,0.9851</t>
+  </si>
+  <si>
+    <t>0.0304,0.0040,0.0038,0.9828</t>
+  </si>
+  <si>
+    <t>0.0054,0.5109,0.9483,0.0068</t>
+  </si>
+  <si>
+    <t>0.9787,0.0080,0.0036,0.0083</t>
+  </si>
+  <si>
+    <t>0.4891,0.5685,0.0291,0.0107</t>
+  </si>
+  <si>
+    <t>0.9751,0.0160,0.0048,0.0050</t>
+  </si>
+  <si>
+    <t>0.8901,0.0960,0.0287,0.0061</t>
+  </si>
+  <si>
+    <t>0.9755,0.0045,0.0017,0.0148</t>
+  </si>
+  <si>
+    <t>0.7511,0.0285,0.0361,0.1871</t>
+  </si>
+  <si>
+    <t>0.9706,0.0055,0.0031,0.0166</t>
+  </si>
+  <si>
+    <t>0.0957,0.7449,0.0865,0.2646</t>
+  </si>
+  <si>
+    <t>0.3950,0.0034,0.0149,0.6517</t>
+  </si>
+  <si>
+    <t>0.7457,0.0130,0.0087,0.2507</t>
+  </si>
+  <si>
+    <t>0.4090,0.6374,0.0429,0.0235</t>
+  </si>
+  <si>
+    <t>0.9293,0.0409,0.0128,0.0171</t>
+  </si>
+  <si>
+    <t>0.6748,0.2725,0.0850,0.0429</t>
+  </si>
+  <si>
+    <t>0.0881,0.7904,0.2060,0.0371</t>
+  </si>
+  <si>
+    <t>0.2090,0.6777,0.1588,0.0115</t>
+  </si>
+  <si>
+    <t>0.5230,0.2474,0.1946,0.0100</t>
+  </si>
+  <si>
+    <t>0.9896,0.0061,0.0015,0.0026</t>
+  </si>
+  <si>
+    <t>0.9847,0.0087,0.0030,0.0038</t>
+  </si>
+  <si>
+    <t>0.9868,0.0071,0.0019,0.0037</t>
+  </si>
+  <si>
+    <t>0.9876,0.0064,0.0024,0.0029</t>
+  </si>
+  <si>
+    <t>0.9932,0.0051,0.0008,0.0011</t>
+  </si>
+  <si>
+    <t>0.9903,0.0060,0.0022,0.0017</t>
+  </si>
+  <si>
+    <t>0.9930,0.0039,0.0007,0.0023</t>
+  </si>
+  <si>
+    <t>0.9894,0.0064,0.0018,0.0025</t>
+  </si>
+  <si>
+    <t>0.3987,0.5711,0.0597,0.0048</t>
+  </si>
+  <si>
+    <t>0.9217,0.0839,0.0123,0.0035</t>
+  </si>
+  <si>
+    <t>0.6355,0.3701,0.0444,0.0092</t>
+  </si>
+  <si>
+    <t>0.2897,0.0701,0.7233,0.0030</t>
+  </si>
+  <si>
+    <t>0.9849,0.0153,0.0024,0.0012</t>
+  </si>
+  <si>
+    <t>0.9459,0.0336,0.0147,0.0083</t>
+  </si>
+  <si>
+    <t>0.9846,0.0165,0.0019,0.0009</t>
+  </si>
+  <si>
+    <t>0.7935,0.2273,0.0282,0.0055</t>
+  </si>
+  <si>
+    <t>0.0297,0.3561,0.8832,0.0113</t>
+  </si>
+  <si>
+    <t>0.9841,0.0182,0.0018,0.0018</t>
+  </si>
+  <si>
+    <t>0.0072,0.0279,0.9816,0.0088</t>
+  </si>
+  <si>
+    <t>0.0069,0.5634,0.9485,0.0078</t>
+  </si>
+  <si>
+    <t>0.0388,0.0314,0.9460,0.0105</t>
+  </si>
+  <si>
+    <t>0.0021,0.1988,0.9865,0.0052</t>
+  </si>
+  <si>
+    <t>0.0169,0.1344,0.9528,0.0052</t>
+  </si>
+  <si>
+    <t>0.0061,0.0190,0.9874,0.0036</t>
+  </si>
+  <si>
+    <t>0.0119,0.1633,0.9662,0.0067</t>
+  </si>
+  <si>
+    <t>0.0865,0.1009,0.8760,0.0074</t>
+  </si>
+  <si>
+    <t>0.0720,0.2611,0.7540,0.0977</t>
+  </si>
+  <si>
+    <t>0.2496,0.5386,0.1421,0.2481</t>
+  </si>
+  <si>
+    <t>0.2048,0.4720,0.3350,0.0211</t>
+  </si>
+  <si>
+    <t>0.2006,0.5302,0.2595,0.0195</t>
+  </si>
+  <si>
+    <t>0.3006,0.4619,0.1848,0.0150</t>
+  </si>
+  <si>
+    <t>0.3436,0.1626,0.5183,0.0237</t>
+  </si>
+  <si>
+    <t>0.4753,0.1147,0.4790,0.0545</t>
+  </si>
+  <si>
+    <t>0.9284,0.0831,0.0116,0.0034</t>
+  </si>
+  <si>
+    <t>0.9618,0.0521,0.0046,0.0020</t>
+  </si>
+  <si>
+    <t>0.9443,0.0776,0.0067,0.0026</t>
+  </si>
+  <si>
+    <t>0.9799,0.0218,0.0036,0.0017</t>
+  </si>
+  <si>
+    <t>0.9095,0.0958,0.0142,0.0034</t>
+  </si>
+  <si>
+    <t>0.1663,0.7569,0.1375,0.0823</t>
+  </si>
+  <si>
+    <t>0.8217,0.0554,0.1035,0.0157</t>
+  </si>
+  <si>
+    <t>0.3451,0.5272,0.1201,0.1380</t>
+  </si>
+  <si>
+    <t>0.4091,0.0747,0.6114,0.0456</t>
+  </si>
+  <si>
+    <t>0.2467,0.2555,0.0758,0.6038</t>
+  </si>
+  <si>
+    <t>0.0038,0.0919,0.9811,0.0087</t>
+  </si>
+  <si>
+    <t>0.0110,0.4666,0.9112,0.0326</t>
+  </si>
+  <si>
+    <t>0.0288,0.3793,0.8884,0.0541</t>
+  </si>
+  <si>
+    <t>0.0216,0.4036,0.9108,0.0133</t>
+  </si>
+  <si>
+    <t>0.0171,0.1283,0.9531,0.0115</t>
+  </si>
+  <si>
+    <t>0.9929,0.0039,0.0008,0.0022</t>
+  </si>
+  <si>
+    <t>0.9888,0.0067,0.0021,0.0020</t>
+  </si>
+  <si>
+    <t>0.9906,0.0081,0.0014,0.0016</t>
+  </si>
+  <si>
+    <t>0.9906,0.0094,0.0013,0.0010</t>
+  </si>
+  <si>
+    <t>0.9882,0.0098,0.0020,0.0017</t>
+  </si>
+  <si>
+    <t>0.9923,0.0056,0.0012,0.0013</t>
+  </si>
+  <si>
+    <t>0.9885,0.0066,0.0022,0.0026</t>
+  </si>
+  <si>
+    <t>0.9890,0.0071,0.0016,0.0024</t>
+  </si>
+  <si>
+    <t>0.1387,0.0579,0.8730,0.0094</t>
+  </si>
+  <si>
+    <t>0.2190,0.5332,0.2202,0.0086</t>
+  </si>
+  <si>
+    <t>0.9573,0.0206,0.0169,0.0053</t>
+  </si>
+  <si>
+    <t>0.0035,0.0248,0.9895,0.0031</t>
+  </si>
+  <si>
+    <t>0.0009,0.0086,0.9910,0.0140</t>
+  </si>
+  <si>
+    <t>0.0130,0.2983,0.9150,0.0174</t>
+  </si>
+  <si>
+    <t>0.0007,0.0101,0.9965,0.0038</t>
+  </si>
+  <si>
+    <t>0.0749,0.2269,0.7798,0.0142</t>
+  </si>
+  <si>
+    <t>0.0010,0.0815,0.9949,0.0019</t>
+  </si>
+  <si>
+    <t>0.0594,0.0825,0.9007,0.0118</t>
+  </si>
+  <si>
+    <t>0.1116,0.4008,0.5747,0.0209</t>
+  </si>
+  <si>
+    <t>0.2989,0.3431,0.4051,0.0275</t>
+  </si>
+  <si>
+    <t>0.1648,0.0325,0.7923,0.0480</t>
+  </si>
+  <si>
+    <t>0.7052,0.0978,0.1594,0.0743</t>
+  </si>
+  <si>
+    <t>0.9859,0.0101,0.0014,0.0037</t>
+  </si>
+  <si>
+    <t>0.9903,0.0068,0.0015,0.0021</t>
+  </si>
+  <si>
+    <t>0.9898,0.0061,0.0018,0.0021</t>
+  </si>
+  <si>
+    <t>0.9919,0.0065,0.0015,0.0012</t>
+  </si>
+  <si>
+    <t>0.9898,0.0090,0.0013,0.0019</t>
+  </si>
+  <si>
+    <t>0.9905,0.0080,0.0017,0.0011</t>
+  </si>
+  <si>
+    <t>0.9914,0.0060,0.0009,0.0019</t>
+  </si>
+  <si>
+    <t>0.9881,0.0098,0.0015,0.0018</t>
+  </si>
+  <si>
+    <t>0.0177,0.2762,0.9254,0.0087</t>
+  </si>
+  <si>
+    <t>0.0110,0.5372,0.9022,0.0057</t>
+  </si>
+  <si>
+    <t>0.0036,0.1358,0.9850,0.0026</t>
+  </si>
+  <si>
+    <t>0.1352,0.4022,0.4662,0.1486</t>
+  </si>
+  <si>
+    <t>0.0103,0.0361,0.9647,0.0183</t>
+  </si>
+  <si>
+    <t>0.0595,0.0482,0.4837,0.5422</t>
+  </si>
+  <si>
+    <t>0.1656,0.2065,0.4451,0.3306</t>
+  </si>
+  <si>
+    <t>0.0131,0.0677,0.9081,0.1006</t>
+  </si>
+  <si>
+    <t>0.6108,0.0480,0.0081,0.4270</t>
+  </si>
+  <si>
+    <t>0.0477,0.0313,0.0058,0.9665</t>
+  </si>
+  <si>
+    <t>0.0086,0.0048,0.0029,0.9925</t>
+  </si>
+  <si>
+    <t>0.0047,0.0039,0.0016,0.9955</t>
+  </si>
+  <si>
+    <t>0.0076,0.0016,0.0004,0.9964</t>
+  </si>
+  <si>
+    <t>0.4331,0.2579,0.0918,0.3851</t>
   </si>
 </sst>
 </file>
@@ -1956,7 +1962,7 @@
         <v>259</v>
       </c>
       <c r="D2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1970,7 +1976,7 @@
         <v>260</v>
       </c>
       <c r="D3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1981,10 +1987,10 @@
         <v>259</v>
       </c>
       <c r="C4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1998,7 +2004,7 @@
         <v>260</v>
       </c>
       <c r="D5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2012,7 +2018,7 @@
         <v>259</v>
       </c>
       <c r="D6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2026,7 +2032,7 @@
         <v>259</v>
       </c>
       <c r="D7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2040,7 +2046,7 @@
         <v>259</v>
       </c>
       <c r="D8" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2054,7 +2060,7 @@
         <v>259</v>
       </c>
       <c r="D9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2068,7 +2074,7 @@
         <v>259</v>
       </c>
       <c r="D10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2082,7 +2088,7 @@
         <v>259</v>
       </c>
       <c r="D11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2096,7 +2102,7 @@
         <v>259</v>
       </c>
       <c r="D12" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2110,7 +2116,7 @@
         <v>259</v>
       </c>
       <c r="D13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2121,10 +2127,10 @@
         <v>259</v>
       </c>
       <c r="C14" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2138,7 +2144,7 @@
         <v>261</v>
       </c>
       <c r="D15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2152,7 +2158,7 @@
         <v>261</v>
       </c>
       <c r="D16" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2166,7 +2172,7 @@
         <v>263</v>
       </c>
       <c r="D17" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2180,7 +2186,7 @@
         <v>259</v>
       </c>
       <c r="D18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2194,7 +2200,7 @@
         <v>262</v>
       </c>
       <c r="D19" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2208,7 +2214,7 @@
         <v>262</v>
       </c>
       <c r="D20" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2222,7 +2228,7 @@
         <v>262</v>
       </c>
       <c r="D21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2236,7 +2242,7 @@
         <v>262</v>
       </c>
       <c r="D22" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2250,7 +2256,7 @@
         <v>262</v>
       </c>
       <c r="D23" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2264,7 +2270,7 @@
         <v>259</v>
       </c>
       <c r="D24" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2278,7 +2284,7 @@
         <v>261</v>
       </c>
       <c r="D25" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2292,7 +2298,7 @@
         <v>261</v>
       </c>
       <c r="D26" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2306,7 +2312,7 @@
         <v>261</v>
       </c>
       <c r="D27" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2320,7 +2326,7 @@
         <v>261</v>
       </c>
       <c r="D28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2334,7 +2340,7 @@
         <v>261</v>
       </c>
       <c r="D29" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2348,7 +2354,7 @@
         <v>261</v>
       </c>
       <c r="D30" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2362,7 +2368,7 @@
         <v>262</v>
       </c>
       <c r="D31" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2376,7 +2382,7 @@
         <v>261</v>
       </c>
       <c r="D32" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2390,7 +2396,7 @@
         <v>261</v>
       </c>
       <c r="D33" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2404,7 +2410,7 @@
         <v>262</v>
       </c>
       <c r="D34" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2418,7 +2424,7 @@
         <v>259</v>
       </c>
       <c r="D35" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2429,10 +2435,10 @@
         <v>259</v>
       </c>
       <c r="C36" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D36" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2446,7 +2452,7 @@
         <v>259</v>
       </c>
       <c r="D37" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2460,7 +2466,7 @@
         <v>262</v>
       </c>
       <c r="D38" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2471,10 +2477,10 @@
         <v>263</v>
       </c>
       <c r="C39" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D39" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2488,7 +2494,7 @@
         <v>261</v>
       </c>
       <c r="D40" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2502,7 +2508,7 @@
         <v>263</v>
       </c>
       <c r="D41" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2516,7 +2522,7 @@
         <v>261</v>
       </c>
       <c r="D42" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2527,10 +2533,10 @@
         <v>263</v>
       </c>
       <c r="C43" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D43" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2541,10 +2547,10 @@
         <v>262</v>
       </c>
       <c r="C44" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D44" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2555,10 +2561,10 @@
         <v>261</v>
       </c>
       <c r="C45" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D45" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2569,10 +2575,10 @@
         <v>259</v>
       </c>
       <c r="C46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2586,7 +2592,7 @@
         <v>262</v>
       </c>
       <c r="D47" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2600,7 +2606,7 @@
         <v>262</v>
       </c>
       <c r="D48" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2614,7 +2620,7 @@
         <v>262</v>
       </c>
       <c r="D49" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2625,10 +2631,10 @@
         <v>261</v>
       </c>
       <c r="C50" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D50" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2642,7 +2648,7 @@
         <v>263</v>
       </c>
       <c r="D51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2656,7 +2662,7 @@
         <v>261</v>
       </c>
       <c r="D52" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2670,7 +2676,7 @@
         <v>261</v>
       </c>
       <c r="D53" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2684,7 +2690,7 @@
         <v>261</v>
       </c>
       <c r="D54" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2698,7 +2704,7 @@
         <v>261</v>
       </c>
       <c r="D55" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2712,7 +2718,7 @@
         <v>259</v>
       </c>
       <c r="D56" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2726,7 +2732,7 @@
         <v>259</v>
       </c>
       <c r="D57" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2740,7 +2746,7 @@
         <v>259</v>
       </c>
       <c r="D58" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2754,7 +2760,7 @@
         <v>261</v>
       </c>
       <c r="D59" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2768,7 +2774,7 @@
         <v>259</v>
       </c>
       <c r="D60" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2782,7 +2788,7 @@
         <v>259</v>
       </c>
       <c r="D61" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -2796,7 +2802,7 @@
         <v>259</v>
       </c>
       <c r="D62" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2810,7 +2816,7 @@
         <v>262</v>
       </c>
       <c r="D63" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2821,10 +2827,10 @@
         <v>261</v>
       </c>
       <c r="C64" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D64" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2838,7 +2844,7 @@
         <v>261</v>
       </c>
       <c r="D65" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2852,7 +2858,7 @@
         <v>263</v>
       </c>
       <c r="D66" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2866,7 +2872,7 @@
         <v>261</v>
       </c>
       <c r="D67" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2880,7 +2886,7 @@
         <v>262</v>
       </c>
       <c r="D68" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2894,7 +2900,7 @@
         <v>262</v>
       </c>
       <c r="D69" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2905,10 +2911,10 @@
         <v>259</v>
       </c>
       <c r="C70" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="D70" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2922,7 +2928,7 @@
         <v>259</v>
       </c>
       <c r="D71" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2936,7 +2942,7 @@
         <v>261</v>
       </c>
       <c r="D72" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2950,7 +2956,7 @@
         <v>263</v>
       </c>
       <c r="D73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2964,7 +2970,7 @@
         <v>263</v>
       </c>
       <c r="D74" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2978,7 +2984,7 @@
         <v>262</v>
       </c>
       <c r="D75" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -2992,7 +2998,7 @@
         <v>262</v>
       </c>
       <c r="D76" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3006,7 +3012,7 @@
         <v>260</v>
       </c>
       <c r="D77" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3020,7 +3026,7 @@
         <v>260</v>
       </c>
       <c r="D78" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3034,7 +3040,7 @@
         <v>260</v>
       </c>
       <c r="D79" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3048,7 +3054,7 @@
         <v>260</v>
       </c>
       <c r="D80" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3062,7 +3068,7 @@
         <v>260</v>
       </c>
       <c r="D81" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3076,7 +3082,7 @@
         <v>260</v>
       </c>
       <c r="D82" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3087,10 +3093,10 @@
         <v>263</v>
       </c>
       <c r="C83" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D83" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3104,7 +3110,7 @@
         <v>263</v>
       </c>
       <c r="D84" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3118,7 +3124,7 @@
         <v>263</v>
       </c>
       <c r="D85" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3132,7 +3138,7 @@
         <v>263</v>
       </c>
       <c r="D86" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3146,7 +3152,7 @@
         <v>263</v>
       </c>
       <c r="D87" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3157,10 +3163,10 @@
         <v>262</v>
       </c>
       <c r="C88" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D88" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3174,7 +3180,7 @@
         <v>259</v>
       </c>
       <c r="D89" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3188,7 +3194,7 @@
         <v>259</v>
       </c>
       <c r="D90" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3202,7 +3208,7 @@
         <v>259</v>
       </c>
       <c r="D91" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3216,7 +3222,7 @@
         <v>259</v>
       </c>
       <c r="D92" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3230,7 +3236,7 @@
         <v>259</v>
       </c>
       <c r="D93" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3244,7 +3250,7 @@
         <v>259</v>
       </c>
       <c r="D94" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3258,7 +3264,7 @@
         <v>259</v>
       </c>
       <c r="D95" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3272,7 +3278,7 @@
         <v>259</v>
       </c>
       <c r="D96" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3286,7 +3292,7 @@
         <v>259</v>
       </c>
       <c r="D97" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3300,7 +3306,7 @@
         <v>259</v>
       </c>
       <c r="D98" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3314,7 +3320,7 @@
         <v>259</v>
       </c>
       <c r="D99" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3328,7 +3334,7 @@
         <v>259</v>
       </c>
       <c r="D100" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3342,7 +3348,7 @@
         <v>259</v>
       </c>
       <c r="D101" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3356,7 +3362,7 @@
         <v>259</v>
       </c>
       <c r="D102" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3370,7 +3376,7 @@
         <v>259</v>
       </c>
       <c r="D103" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3384,7 +3390,7 @@
         <v>259</v>
       </c>
       <c r="D104" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3398,7 +3404,7 @@
         <v>261</v>
       </c>
       <c r="D105" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3412,7 +3418,7 @@
         <v>261</v>
       </c>
       <c r="D106" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3423,10 +3429,10 @@
         <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D107" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3440,7 +3446,7 @@
         <v>261</v>
       </c>
       <c r="D108" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3454,7 +3460,7 @@
         <v>262</v>
       </c>
       <c r="D109" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3468,7 +3474,7 @@
         <v>262</v>
       </c>
       <c r="D110" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3479,10 +3485,10 @@
         <v>262</v>
       </c>
       <c r="C111" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D111" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3493,10 +3499,10 @@
         <v>262</v>
       </c>
       <c r="C112" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D112" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -3510,7 +3516,7 @@
         <v>262</v>
       </c>
       <c r="D113" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -3524,7 +3530,7 @@
         <v>262</v>
       </c>
       <c r="D114" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -3535,10 +3541,10 @@
         <v>262</v>
       </c>
       <c r="C115" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D115" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -3549,10 +3555,10 @@
         <v>259</v>
       </c>
       <c r="C116" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D116" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -3566,7 +3572,7 @@
         <v>261</v>
       </c>
       <c r="D117" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -3580,7 +3586,7 @@
         <v>262</v>
       </c>
       <c r="D118" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -3591,10 +3597,10 @@
         <v>261</v>
       </c>
       <c r="C119" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D119" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -3605,10 +3611,10 @@
         <v>262</v>
       </c>
       <c r="C120" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D120" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -3622,7 +3628,7 @@
         <v>262</v>
       </c>
       <c r="D121" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -3636,7 +3642,7 @@
         <v>262</v>
       </c>
       <c r="D122" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -3650,7 +3656,7 @@
         <v>262</v>
       </c>
       <c r="D123" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -3664,7 +3670,7 @@
         <v>262</v>
       </c>
       <c r="D124" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -3678,7 +3684,7 @@
         <v>262</v>
       </c>
       <c r="D125" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -3692,7 +3698,7 @@
         <v>259</v>
       </c>
       <c r="D126" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -3706,7 +3712,7 @@
         <v>259</v>
       </c>
       <c r="D127" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -3720,7 +3726,7 @@
         <v>259</v>
       </c>
       <c r="D128" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -3734,7 +3740,7 @@
         <v>259</v>
       </c>
       <c r="D129" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -3748,7 +3754,7 @@
         <v>259</v>
       </c>
       <c r="D130" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -3762,7 +3768,7 @@
         <v>259</v>
       </c>
       <c r="D131" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -3776,7 +3782,7 @@
         <v>259</v>
       </c>
       <c r="D132" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -3790,7 +3796,7 @@
         <v>259</v>
       </c>
       <c r="D133" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -3804,7 +3810,7 @@
         <v>259</v>
       </c>
       <c r="D134" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -3818,7 +3824,7 @@
         <v>259</v>
       </c>
       <c r="D135" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -3832,7 +3838,7 @@
         <v>263</v>
       </c>
       <c r="D136" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -3846,7 +3852,7 @@
         <v>263</v>
       </c>
       <c r="D137" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -3857,10 +3863,10 @@
         <v>261</v>
       </c>
       <c r="C138" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D138" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -3874,7 +3880,7 @@
         <v>261</v>
       </c>
       <c r="D139" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -3888,7 +3894,7 @@
         <v>259</v>
       </c>
       <c r="D140" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -3902,7 +3908,7 @@
         <v>259</v>
       </c>
       <c r="D141" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -3916,7 +3922,7 @@
         <v>261</v>
       </c>
       <c r="D142" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -3927,10 +3933,10 @@
         <v>259</v>
       </c>
       <c r="C143" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D143" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -3944,7 +3950,7 @@
         <v>260</v>
       </c>
       <c r="D144" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -3958,7 +3964,7 @@
         <v>260</v>
       </c>
       <c r="D145" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -3972,7 +3978,7 @@
         <v>260</v>
       </c>
       <c r="D146" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -3986,7 +3992,7 @@
         <v>260</v>
       </c>
       <c r="D147" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4000,7 +4006,7 @@
         <v>263</v>
       </c>
       <c r="D148" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4014,7 +4020,7 @@
         <v>259</v>
       </c>
       <c r="D149" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4025,10 +4031,10 @@
         <v>262</v>
       </c>
       <c r="C150" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D150" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4042,7 +4048,7 @@
         <v>259</v>
       </c>
       <c r="D151" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4056,7 +4062,7 @@
         <v>259</v>
       </c>
       <c r="D152" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4070,7 +4076,7 @@
         <v>259</v>
       </c>
       <c r="D153" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4084,7 +4090,7 @@
         <v>259</v>
       </c>
       <c r="D154" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4098,7 +4104,7 @@
         <v>259</v>
       </c>
       <c r="D155" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4112,7 +4118,7 @@
         <v>262</v>
       </c>
       <c r="D156" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4126,7 +4132,7 @@
         <v>260</v>
       </c>
       <c r="D157" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4140,7 +4146,7 @@
         <v>259</v>
       </c>
       <c r="D158" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4154,7 +4160,7 @@
         <v>262</v>
       </c>
       <c r="D159" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4168,7 +4174,7 @@
         <v>259</v>
       </c>
       <c r="D160" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4182,7 +4188,7 @@
         <v>259</v>
       </c>
       <c r="D161" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4196,7 +4202,7 @@
         <v>262</v>
       </c>
       <c r="D162" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4207,10 +4213,10 @@
         <v>259</v>
       </c>
       <c r="C163" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D163" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4224,7 +4230,7 @@
         <v>259</v>
       </c>
       <c r="D164" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4238,7 +4244,7 @@
         <v>259</v>
       </c>
       <c r="D165" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4252,7 +4258,7 @@
         <v>259</v>
       </c>
       <c r="D166" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4266,7 +4272,7 @@
         <v>259</v>
       </c>
       <c r="D167" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4280,7 +4286,7 @@
         <v>259</v>
       </c>
       <c r="D168" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4294,7 +4300,7 @@
         <v>259</v>
       </c>
       <c r="D169" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4308,7 +4314,7 @@
         <v>259</v>
       </c>
       <c r="D170" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4322,7 +4328,7 @@
         <v>259</v>
       </c>
       <c r="D171" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4336,7 +4342,7 @@
         <v>259</v>
       </c>
       <c r="D172" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4347,10 +4353,10 @@
         <v>259</v>
       </c>
       <c r="C173" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D173" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4364,7 +4370,7 @@
         <v>259</v>
       </c>
       <c r="D174" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4378,7 +4384,7 @@
         <v>259</v>
       </c>
       <c r="D175" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4389,10 +4395,10 @@
         <v>261</v>
       </c>
       <c r="C176" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D176" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4406,7 +4412,7 @@
         <v>259</v>
       </c>
       <c r="D177" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4420,7 +4426,7 @@
         <v>259</v>
       </c>
       <c r="D178" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4434,7 +4440,7 @@
         <v>259</v>
       </c>
       <c r="D179" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4448,7 +4454,7 @@
         <v>259</v>
       </c>
       <c r="D180" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4462,7 +4468,7 @@
         <v>261</v>
       </c>
       <c r="D181" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4476,7 +4482,7 @@
         <v>259</v>
       </c>
       <c r="D182" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4490,7 +4496,7 @@
         <v>261</v>
       </c>
       <c r="D183" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4504,7 +4510,7 @@
         <v>263</v>
       </c>
       <c r="D184" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -4518,7 +4524,7 @@
         <v>261</v>
       </c>
       <c r="D185" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -4532,7 +4538,7 @@
         <v>261</v>
       </c>
       <c r="D186" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -4546,7 +4552,7 @@
         <v>261</v>
       </c>
       <c r="D187" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -4560,7 +4566,7 @@
         <v>261</v>
       </c>
       <c r="D188" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -4574,7 +4580,7 @@
         <v>261</v>
       </c>
       <c r="D189" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -4585,10 +4591,10 @@
         <v>259</v>
       </c>
       <c r="C190" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D190" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -4602,7 +4608,7 @@
         <v>261</v>
       </c>
       <c r="D191" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -4613,10 +4619,10 @@
         <v>259</v>
       </c>
       <c r="C192" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D192" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -4627,10 +4633,10 @@
         <v>261</v>
       </c>
       <c r="C193" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D193" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -4641,10 +4647,10 @@
         <v>261</v>
       </c>
       <c r="C194" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D194" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -4655,10 +4661,10 @@
         <v>261</v>
       </c>
       <c r="C195" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D195" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -4669,10 +4675,10 @@
         <v>259</v>
       </c>
       <c r="C196" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D196" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -4683,10 +4689,10 @@
         <v>259</v>
       </c>
       <c r="C197" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D197" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -4700,7 +4706,7 @@
         <v>259</v>
       </c>
       <c r="D198" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -4714,7 +4720,7 @@
         <v>259</v>
       </c>
       <c r="D199" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -4728,7 +4734,7 @@
         <v>259</v>
       </c>
       <c r="D200" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -4742,7 +4748,7 @@
         <v>259</v>
       </c>
       <c r="D201" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -4756,7 +4762,7 @@
         <v>259</v>
       </c>
       <c r="D202" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -4770,7 +4776,7 @@
         <v>262</v>
       </c>
       <c r="D203" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -4784,7 +4790,7 @@
         <v>259</v>
       </c>
       <c r="D204" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -4795,10 +4801,10 @@
         <v>259</v>
       </c>
       <c r="C205" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D205" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -4812,7 +4818,7 @@
         <v>261</v>
       </c>
       <c r="D206" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -4823,10 +4829,10 @@
         <v>259</v>
       </c>
       <c r="C207" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D207" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -4840,7 +4846,7 @@
         <v>261</v>
       </c>
       <c r="D208" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -4854,7 +4860,7 @@
         <v>261</v>
       </c>
       <c r="D209" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -4868,7 +4874,7 @@
         <v>261</v>
       </c>
       <c r="D210" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -4882,7 +4888,7 @@
         <v>261</v>
       </c>
       <c r="D211" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -4896,7 +4902,7 @@
         <v>261</v>
       </c>
       <c r="D212" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -4910,7 +4916,7 @@
         <v>259</v>
       </c>
       <c r="D213" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -4924,7 +4930,7 @@
         <v>259</v>
       </c>
       <c r="D214" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -4938,7 +4944,7 @@
         <v>259</v>
       </c>
       <c r="D215" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -4952,7 +4958,7 @@
         <v>259</v>
       </c>
       <c r="D216" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -4966,7 +4972,7 @@
         <v>259</v>
       </c>
       <c r="D217" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -4980,7 +4986,7 @@
         <v>259</v>
       </c>
       <c r="D218" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -4994,7 +5000,7 @@
         <v>259</v>
       </c>
       <c r="D219" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5008,7 +5014,7 @@
         <v>259</v>
       </c>
       <c r="D220" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5022,7 +5028,7 @@
         <v>261</v>
       </c>
       <c r="D221" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5036,7 +5042,7 @@
         <v>262</v>
       </c>
       <c r="D222" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5050,7 +5056,7 @@
         <v>259</v>
       </c>
       <c r="D223" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5064,7 +5070,7 @@
         <v>261</v>
       </c>
       <c r="D224" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5078,7 +5084,7 @@
         <v>261</v>
       </c>
       <c r="D225" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5092,7 +5098,7 @@
         <v>261</v>
       </c>
       <c r="D226" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5106,7 +5112,7 @@
         <v>261</v>
       </c>
       <c r="D227" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5120,7 +5126,7 @@
         <v>261</v>
       </c>
       <c r="D228" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5134,7 +5140,7 @@
         <v>261</v>
       </c>
       <c r="D229" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5148,7 +5154,7 @@
         <v>261</v>
       </c>
       <c r="D230" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5159,10 +5165,10 @@
         <v>261</v>
       </c>
       <c r="C231" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D231" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5173,10 +5179,10 @@
         <v>259</v>
       </c>
       <c r="C232" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D232" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5187,10 +5193,10 @@
         <v>259</v>
       </c>
       <c r="C233" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D233" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5204,7 +5210,7 @@
         <v>259</v>
       </c>
       <c r="D234" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5218,7 +5224,7 @@
         <v>259</v>
       </c>
       <c r="D235" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5232,7 +5238,7 @@
         <v>259</v>
       </c>
       <c r="D236" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5246,7 +5252,7 @@
         <v>259</v>
       </c>
       <c r="D237" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5260,7 +5266,7 @@
         <v>259</v>
       </c>
       <c r="D238" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5274,7 +5280,7 @@
         <v>259</v>
       </c>
       <c r="D239" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5288,7 +5294,7 @@
         <v>259</v>
       </c>
       <c r="D240" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5302,7 +5308,7 @@
         <v>259</v>
       </c>
       <c r="D241" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5316,7 +5322,7 @@
         <v>259</v>
       </c>
       <c r="D242" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5330,7 +5336,7 @@
         <v>261</v>
       </c>
       <c r="D243" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5341,10 +5347,10 @@
         <v>261</v>
       </c>
       <c r="C244" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D244" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5355,10 +5361,10 @@
         <v>261</v>
       </c>
       <c r="C245" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D245" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5369,10 +5375,10 @@
         <v>261</v>
       </c>
       <c r="C246" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D246" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5386,7 +5392,7 @@
         <v>261</v>
       </c>
       <c r="D247" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -5397,10 +5403,10 @@
         <v>261</v>
       </c>
       <c r="C248" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D248" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -5411,10 +5417,10 @@
         <v>261</v>
       </c>
       <c r="C249" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D249" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -5428,7 +5434,7 @@
         <v>261</v>
       </c>
       <c r="D250" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -5439,10 +5445,10 @@
         <v>259</v>
       </c>
       <c r="C251" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D251" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -5456,7 +5462,7 @@
         <v>260</v>
       </c>
       <c r="D252" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -5470,7 +5476,7 @@
         <v>260</v>
       </c>
       <c r="D253" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -5484,7 +5490,7 @@
         <v>260</v>
       </c>
       <c r="D254" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -5498,7 +5504,7 @@
         <v>260</v>
       </c>
       <c r="D255" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -5509,10 +5515,10 @@
         <v>259</v>
       </c>
       <c r="C256" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D256" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
   </sheetData>

</xml_diff>